<commit_message>
add issues 25 and 26
</commit_message>
<xml_diff>
--- a/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
+++ b/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\troyr\Documents\Troy's\AI\Andrews_Driving_Service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59206B91-8276-4B0E-8CE6-C5ABBE92720E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA326316-B058-42A4-8DBB-3569287C1D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="142">
   <si>
     <t>Entry #</t>
   </si>
@@ -413,6 +413,39 @@
   </si>
   <si>
     <t>Deliberate "good enough for now" choices deserve their own record, distinct from breadth-capture log entries.</t>
+  </si>
+  <si>
+    <t>Aug 14 2026</t>
+  </si>
+  <si>
+    <t>Advisory session (post-Rung-2-attempt-1)</t>
+  </si>
+  <si>
+    <t>Migrating the Goal Card, Issues Log, deferred-decisions doc, and restart doc into andrews-driving-services/agentic-loop-ops/ (done for git-history and convenience reasons) gave the /goal-invoking Claude Code session — and worker, business-analyst, and qa, all running in the same repo — unrestricted Read/Glob/Bash access to everything in that directory. That included the Answer Key's literal external path, stated in plain text in three places in the Goal Card, and the full history of every prior rung's turn counts and wall-clock times.</t>
+  </si>
+  <si>
+    <t>The migration was made for good reasons — real git version history instead of manual _vN filename suffixes, one authoritative copy readable by any session with repo access — but without tracing what else in the architecture would gain reach to the new directory. It reopened the exact isolation problem Entries 9-11 already closed once (worker/business-analyst must never have a reachable path to the Answer Key), and separately contaminated clean rung-to-rung measurement, since the invoking session could now read its own prior results.</t>
+  </si>
+  <si>
+    <t>All four files relocated to troy-kb (a separate, personal repo the Desktop /goal session never touches), and agentic-loop-ops/ fully reverted out of andrews-driving-services (PR #5). Physical absence, not a permission rule.</t>
+  </si>
+  <si>
+    <t>Two, tied together. First, the one already familiar from the Answer Key's own history: isolation by withholding information beats isolation by permission rule — a rule can be misconfigured or misbehave; a file that isn't reachable can't. Second, and arguably the more important one this time: the decision to co-locate these docs inside andrews-driving-services in the first place was made without knowing a Claude Code session could hold two repositories open at once. Absent that knowledge, keeping everything in one repo felt like the only real option. Once the multi-repo capability was actually verified live, the constraint that drove the original choice simply stopped being true. An architectural decision is only as good as the toolset knowledge available when it's made — worth checking what's actually possible before assuming a constraint is real.</t>
+  </si>
+  <si>
+    <t>Rung 2 attempt #2 (pre-fire)</t>
+  </si>
+  <si>
+    <t>Firing Rung 2 attempt #2 with the (then-current) v7 /goal command text failed outright: "Goal condition is limited to 4000 characters (got 4323)." Nothing before this point had ever come close to that limit.</t>
+  </si>
+  <si>
+    <t>v6 and v7 both added real, substantive text directly into the pasteable /goal command block (the Glob/Read preflight fallback, then the Explicit Hard-Stop STOP clause) without either revision checking the block's total length against any known ceiling — because no such ceiling had ever been hit before.</t>
+  </si>
+  <si>
+    <t>Tightened the command text to 3,724 characters — cut wordiness only, no rule dropped — and folded it into Goal Card v8.</t>
+  </si>
+  <si>
+    <t>A command text that grows via incremental, individually-reasonable additions can cross a hard platform limit with no warning until the exact moment it's fired — worth a rough length gut-check whenever a revision adds prose to that specific block, not just after something rejects it.</t>
   </si>
 </sst>
 </file>
@@ -432,11 +465,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -797,7 +832,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -806,7 +841,7 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="55" customWidth="1"/>
-    <col min="7" max="9" width="39.21875" customWidth="1"/>
+    <col min="7" max="9" width="40.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -838,7 +873,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -865,7 +900,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="69" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -892,7 +927,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -919,7 +954,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -946,7 +981,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="69" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -973,7 +1008,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1000,7 +1035,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1027,7 +1062,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1054,7 +1089,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1081,7 +1116,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1108,7 +1143,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1135,7 +1170,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1164,7 +1199,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1191,7 +1226,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1218,7 +1253,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1245,7 +1280,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1274,7 +1309,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1303,7 +1338,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1332,7 +1367,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1361,7 +1396,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="151.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="207" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1504,16 +1539,74 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
+    <row r="26" spans="1:9" ht="289.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="183.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add 5 hard hitting issues but more entries coming
</commit_message>
<xml_diff>
--- a/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
+++ b/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\troyr\Documents\Troy's\AI\Andrews_Driving_Service\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\troyr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA326316-B058-42A4-8DBB-3569287C1D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD19FC6-2086-450E-BF46-BBE71631A347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="166">
   <si>
     <t>Entry #</t>
   </si>
@@ -446,6 +446,78 @@
   </si>
   <si>
     <t>A command text that grows via incremental, individually-reasonable additions can cross a hard platform limit with no warning until the exact moment it's fired — worth a rough length gut-check whenever a revision adds prose to that specific block, not just after something rejects it.</t>
+  </si>
+  <si>
+    <t>Aug 15 2026</t>
+  </si>
+  <si>
+    <t>Rung 3, row 4 (Venue Number 16)</t>
+  </si>
+  <si>
+    <t>Worker passed a markdown-formatted link ([text](url)) verbatim into a WebFetch/path argument while researching Glass House Winery's PDF menu. Something downstream interpreted the whole bracket-and-backslash string as a Windows file path relative to the repo root, producing a mangled path that Claude Code's own path-safety heuristic correctly flagged. Troy declined it, and the row 4 worker got killed outright as a direct consequence — the first worker-kill of the session.</t>
+  </si>
+  <si>
+    <t>Neither worker.md nor business-analyst.md ever instructed extracting the bare URL before a WebFetch call — a markdown link copied straight out of search-result text was passed through as-is.</t>
+  </si>
+  <si>
+    <t>Added an explicit instruction to both subagent files: always extract the bare URL first, never pass markdown link syntax through verbatim, regardless of the form a source presented it in.</t>
+  </si>
+  <si>
+    <t>A malformed argument can masquerade as a suspicious path and trigger a legitimate security check, costing a killed subagent — worth guarding the argument-construction step directly rather than relying on the safety heuristic to keep catching it after the fact.</t>
+  </si>
+  <si>
+    <t>Rung 5, row 2 (Moss Vineyards)</t>
+  </si>
+  <si>
+    <t>Business-analyst's Bash calls during its first-ever consultation (--help, dump-audit-log, dump-data-dictionary, read-row) all used an absolute-path invocation shape (python C:/workspaces/.../scripts/ads_xlsx_tool.py ...) that the Bash PreToolUse hook's exact-prefix check didn't recognize, so every call fell through to a live Allow-once prompt.</t>
+  </si>
+  <si>
+    <t>The hook's sanctioned-command check was an exact-prefix tuple built from worker's known invocation shapes; it never anticipated bare python + absolute script path — a shape business-analyst used consistently but worker never had.</t>
+  </si>
+  <si>
+    <t>Replaced the exact-prefix check with real shell-aware tokenization (shlex with punctuation_chars) that recognizes the sanctioned script by its trailing path regardless of interpreter or path form, and rejects command chaining/redirection anywhere after the script argument. The logic lives in a dedicated file, .claude/hooks/check_sanctioned_bash.py, rather than an inline one-liner, so it stays reviewable as normal Python. Verified against real invocation shapes and adversarial cases — including chaining attempts and a legitimate pipe-delimited Source References value — before deploying.</t>
+  </si>
+  <si>
+    <t>An exact-prefix allowlist is only as complete as the shapes you've actually observed — matching on the invariant that actually matters (which script is being invoked) holds up better than enumerating every way of expressing it.</t>
+  </si>
+  <si>
+    <t>The Audit Log's Rung column was found to carry no real information — every existing entry read "1 row" regardless of the actual rung it came from, even though business-analyst.md described it as meant to record the current rung's true size.</t>
+  </si>
+  <si>
+    <t>Nothing in the architecture actually threads the rung's true row count down to worker or business-analyst — worker only ever knows it's handling exactly one row, by design, per its own per-invocation scope, and that was the only "row count" fact that ever made it into the field.</t>
+  </si>
+  <si>
+    <t>Removed the Rung column entirely, rather than fixing it, on the reasoning that it was the wrong column to have committed to in the first place — Timestamp already places an entry in temporal context well enough for Troy's purposes, and making Rung genuinely accurate would require new plumbing in every future /goal invocation just to feed one field. Removed from the schema: scripts/ads_xlsx_tool.py (docstring, argparse, AUDIT_LOG_COLUMNS, the row it writes), business-analyst.md (invocation example and column list, renumbered), and the Goal Card (v9 — the terminology table's description dropped the column-count language too, so it won't need editing again the next time the schema changes). Troy handled the live audit_log.xlsx column deletion directly in Excel.</t>
+  </si>
+  <si>
+    <t>A documented field that requires plumbing nothing in the architecture actually supplies will quietly collapse to whatever's locally available instead — and sometimes the right fix isn't repairing the field, it's recognizing another field already does that job well enough.</t>
+  </si>
+  <si>
+    <t>Business-analyst had to work substantially harder than the geographic fork itself required to discern the correct value format for the County field — bare county name, no "County" suffix, (city) appended only for independent cities. The Data Dictionary didn't state this convention anywhere; business-analyst only found it by discovering and reading ADS_ListMaker_Rules.md, a file outside the loop's normal CONTEXT, as a side effect of its broader research into the Moss Vineyards county fork.</t>
+  </si>
+  <si>
+    <t>The bare-name convention is real and deliberate — it's baked into ListMaker's own 26-county scope list — but it was never carried forward into the Data Dictionary or Operating Guide when RowBuilder's process split off from ListMaker's. The two docs drifted apart on this one point.</t>
+  </si>
+  <si>
+    <t>Data Dictionary's County field entry updated to state the convention explicitly — plain county name, no "County" word, (city) suffix reserved for independent cities — with worked examples. Troy also went back and corrected existing County values already in the Master to comply, better late than never. Both edits made directly in Excel.</t>
+  </si>
+  <si>
+    <t>A conflicting-sources judgment call and a missing value-formatting convention can surface together inside the same fork, but they're two different kinds of gaps — resolving which county was correct didn't also guarantee the format of the answer was documented anywhere worker or business-analyst could reliably find it.</t>
+  </si>
+  <si>
+    <t>Rung 5, row 5 (Reynard Florence)</t>
+  </si>
+  <si>
+    <t>Worker caught a live instance of the $ shell-expansion bug in a Source References field value during a pricing-fork resolution — not a price field, even though the only existing documentation (the Operating Guide's Price Field Convention) framed the underlying mechanical problem as specific to price fields.</t>
+  </si>
+  <si>
+    <t>The Price Field Convention (added in v3.4, after the original Rung 1B incident) correctly explained the shell mechanics of why a literal $ breaks a write command, but scoped that explanation narrowly to price fields, since that was the only place the bug had been observed at the time. The mechanism is actually a property of how any value reaches ads_xlsx_tool.py, not of what the field means.</t>
+  </si>
+  <si>
+    <t>Operating Guide bumped to v3.5. The price-specific formatting rule (plain numbers, no currency symbol) is unchanged; a new clause broadens the shell-escaping explanation to state plainly that a literal $ in any field's value can trigger the same problem, citing the Source References instance as confirmation it isn't price-specific. Data Dictionary intentionally left untouched — its price-specific note there still correctly applies only to price fields.</t>
+  </si>
+  <si>
+    <t>A documented workaround discovered from one specific incident can get scoped too narrowly to that incident's context — the underlying mechanism mattered more than the field it happened to be caught in.</t>
   </si>
 </sst>
 </file>
@@ -515,7 +587,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -529,7 +601,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -832,7 +903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -873,7 +944,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -900,7 +971,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="69" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -927,7 +998,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -954,7 +1025,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -981,7 +1052,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="69" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1008,7 +1079,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1035,7 +1106,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1062,7 +1133,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1089,7 +1160,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1116,7 +1187,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1143,7 +1214,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1170,7 +1241,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1199,7 +1270,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1226,7 +1297,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1253,7 +1324,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1280,7 +1351,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1309,7 +1380,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1338,7 +1409,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1367,7 +1438,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="96.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1396,7 +1467,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="207" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="207" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1539,7 +1610,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="289.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="289.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1597,16 +1668,150 @@
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
+    <row r="28" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="220.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="276" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="151.80000000000001" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>165</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add couple more items to Issues Log
</commit_message>
<xml_diff>
--- a/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
+++ b/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\troyr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD19FC6-2086-450E-BF46-BBE71631A347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BBF3118-EA3D-4679-9F77-665AAE69FDDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="177">
   <si>
     <t>Entry #</t>
   </si>
@@ -518,6 +518,39 @@
   </si>
   <si>
     <t>A documented workaround discovered from one specific incident can get scoped too narrowly to that incident's context — the underlying mechanism mattered more than the field it happened to be caught in.</t>
+  </si>
+  <si>
+    <t>Rung 5 (observed); Rung 5B retest cycle (fix designed, then deferred)</t>
+  </si>
+  <si>
+    <t>virginiawine.org reliably returns 403 on direct WebFetch (bot-detection), observed repeatedly across venues in Rung 5 and confirmed live by Troy watching subsequent runs.</t>
+  </si>
+  <si>
+    <t>Not applicable — this is an observed platform/domain behavior, not a defect.</t>
+  </si>
+  <si>
+    <t>Deferred. A full fix was designed, drafted, and verified working, then deliberately not shipped — see deferred-design-decisions_ads-agentic-loop.md, Decision #3, for the full reasoning and revisit trigger.</t>
+  </si>
+  <si>
+    <t>A fully designed and verified fix doesn't have to ship just because it's ready.</t>
+  </si>
+  <si>
+    <t>Aug 16 2026 (observed Rung 5, Aug 15)</t>
+  </si>
+  <si>
+    <t>Rung 5 (business-analyst pricing and county fork resolutions)</t>
+  </si>
+  <si>
+    <t>Troy observed business-analyst investing heavy effort — multiple sources, many tool calls — resolving forks that didn't all seem to warrant it equally, pricing in particular.</t>
+  </si>
+  <si>
+    <t>Not applicable — an observed effort/stakes mismatch, not a defect.</t>
+  </si>
+  <si>
+    <t>Deferred deliberately; today's priority is infrastructure-hardening toward a supervised, unattended run. See deferred-design-decisions_ads-agentic-loop.md, Decision #4, for the full reasoning and revisit trigger.</t>
+  </si>
+  <si>
+    <t>Not every observed inefficiency needs fixing in the cycle it's noticed in.</t>
   </si>
 </sst>
 </file>
@@ -903,7 +936,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1668,7 +1701,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -1697,7 +1730,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="220.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="220.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -1726,7 +1759,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="276" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="276" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -1755,7 +1788,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1784,7 +1817,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="151.80000000000001" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" ht="151.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -1811,6 +1844,64 @@
       </c>
       <c r="I32" s="4" t="s">
         <v>165</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="69" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
+        <v>33</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add issues to issues log from Rung 6 and 7 fixes
</commit_message>
<xml_diff>
--- a/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
+++ b/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\troyr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BBF3118-EA3D-4679-9F77-665AAE69FDDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25669F7C-D400-4CE3-A7C0-8CBFD309D951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="195">
   <si>
     <t>Entry #</t>
   </si>
@@ -551,6 +551,60 @@
   </si>
   <si>
     <t>Not every observed inefficiency needs fixing in the cycle it's noticed in.</t>
+  </si>
+  <si>
+    <t>Aug 17 2026</t>
+  </si>
+  <si>
+    <t>Rung 6 row 25 (Basic City Beer Co.); Rung 7 row 92-acres</t>
+  </si>
+  <si>
+    <t>Process-Discipline / Architecture</t>
+  </si>
+  <si>
+    <t>Worker tried to peek at a completed row for formatting reference twice: Rung 6 guessed slug 'pippin-hill' wrapped in a malformed Bash command (command substitution + a Windows-incompatible redirect) that tripped a live permission prompt; Rung 7's 92-acres made a second, cleaner guess that just failed.</t>
+  </si>
+  <si>
+    <t>Worker reached for an unsanctioned capability instead of treating the missing reference-row path as a stop-and-report tool-capability gap; no sanctioned way to see a reference row existed at all.</t>
+  </si>
+  <si>
+    <t>Rather than reinforce the stop-and-report prohibition (a fix drafted in PR #9, closed unmerged - it would have become self-contradictory the moment a sanctioned capability shipped, and the prohibition itself had a 0-for-2 track record across both observed occurrences), built a sanctioned sample-reference-row action (Venue Number 3, slug mountain-vine, Troy's chosen example), with a documented fallback to the other five pre-completed rows. Shipped in PR #10. Deferred Decision #5 reversed.</t>
+  </si>
+  <si>
+    <t>When a prohibition-based fix and a legitimate underlying need collide, check whether granting the capability closes the gap more reliably than reinforcing the prohibition - especially once the prohibition has already shown it doesn't reliably hold.</t>
+  </si>
+  <si>
+    <t>Rung 7, great-valley-farm and bluestone (Days/Hours, Full Operating Hours fields)</t>
+  </si>
+  <si>
+    <t>Four live permission prompts across two rows: worker used $(printf ...) command substitution, then ANSI-C $'...' quoting, to embed a required CHAR(10) line break in --value.</t>
+  </si>
+  <si>
+    <t>The Data Dictionary's line-break convention for these two fields had no sanctioned mechanism in write-field to satisfy with a literal argument.</t>
+  </si>
+  <si>
+    <t>write-field now converts a literal \n in --value to a real CHAR(10) before writing. Shipped in PR #10.</t>
+  </si>
+  <si>
+    <t>A permission-prompt pattern that looks structurally identical to another finding can need the opposite fix - this one traced to a legitimate documented data requirement, so the fix was "build the capability," not "tighten the rule."</t>
+  </si>
+  <si>
+    <t>Aug 20 2026</t>
+  </si>
+  <si>
+    <t>Discovered during Entry 35's fix implementation (advisory session, Aug 20)</t>
+  </si>
+  <si>
+    <t>While implementing Entry 35's fix, found write-field never sets wrap_text on cells it writes, though the Data Dictionary states these cells "must/will have wrap_text enabled." The pre-completed rows (2-7) have it set; actual worker-written rows don't.</t>
+  </si>
+  <si>
+    <t>write-field only ever touches a cell's value, never its formatting - never in scope for any prior fix.</t>
+  </si>
+  <si>
+    <t>Declined. Troy's explicit call: doesn't care that these cells lack wrap_text, and doesn't want it added now - possibly ever. A single manual formatting pass across the whole sheet at final completion is the intended remedy, not per-row automation.</t>
+  </si>
+  <si>
+    <t>A gap discovered adjacent to a fix already in progress doesn't have to be fixed just because it's adjacent - a one-time manual cleanup at project completion can be the more sensible remedy than automating every intermediate row..</t>
   </si>
 </sst>
 </file>
@@ -936,7 +990,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1846,7 +1900,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="69" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -1875,7 +1929,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -1902,6 +1956,93 @@
       </c>
       <c r="I34" s="4" t="s">
         <v>176</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add issue 37 to issues log
</commit_message>
<xml_diff>
--- a/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
+++ b/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\troyr\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspaces\troy-kb\projects\ads-agent-ops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25669F7C-D400-4CE3-A7C0-8CBFD309D951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE2030D-5777-425F-996D-6814FE331CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="201">
   <si>
     <t>Entry #</t>
   </si>
@@ -605,6 +605,24 @@
   </si>
   <si>
     <t>A gap discovered adjacent to a fix already in progress doesn't have to be fixed just because it's adjacent - a one-time manual cleanup at project completion can be the more sensible remedy than automating every intermediate row..</t>
+  </si>
+  <si>
+    <t>Rung 8A, rows 90 (blue-shepherd) and 91 (bold-rock-barrel-barn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Tooling-Environment / Architecture</t>
+  </si>
+  <si>
+    <t>Bash's actual working directory resolved to the repo's parent folder instead of the repo root — a documented Claude Code Desktop bug on Windows (GitHub issue #52165). qa hit this on both rows and improvised two different unsanctioned workarounds: row 90 used a banned cd ... &amp;&amp; prefix, row 91 used an unquoted absolute Windows path that the shell's own backslash-escaping rules mangled into an unrecognizable filename, requiring a second self-correction to forward slashes. Separately, the orchestrator had explicitly told qa to "proceed however necessary" on first hitting the bug, rather than treating it as the tool-capability-gap stop-and-report case already required.</t>
+  </si>
+  <si>
+    <t>The existing missing-file Preflight check (via Read/Glob) doesn't verify Bash's own working directory — Read/Glob can resolve correctly even when Bash's cwd is wrong, so Preflight passed while the actual failure mode went undetected until subagents started running.</t>
+  </si>
+  <si>
+    <t>Goal Card v11 adds an independent Preflight check confirming Bash is rooted at the repo (a harmless --help call to the sanctioned script), hard-stopping immediately if not. Shipped via troy-kb PR #4.</t>
+  </si>
+  <si>
+    <t>A preflight check that verifies something through one tool (Read/Glob) doesn't verify the same thing for a different tool (Bash) that does the real work — check the actual mechanism that matters, not a proxy for it.</t>
   </si>
 </sst>
 </file>
@@ -990,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -2045,6 +2063,35 @@
         <v>194</v>
       </c>
     </row>
+    <row r="38" spans="1:9" ht="179.4" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>37</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add 4 new issues from Rung 8B execution
</commit_message>
<xml_diff>
--- a/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
+++ b/projects/ads-agent-ops/AgenticLoop_IssuesLog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspaces\troy-kb\projects\ads-agent-ops\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\troyr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE2030D-5777-425F-996D-6814FE331CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_307562CDD433AB350E64AB9A1E6A0D6179FA5DF6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="222">
   <si>
     <t>Entry #</t>
   </si>
@@ -623,6 +623,69 @@
   </si>
   <si>
     <t>A preflight check that verifies something through one tool (Read/Glob) doesn't verify the same thing for a different tool (Bash) that does the real work — check the actual mechanism that matters, not a proxy for it.</t>
+  </si>
+  <si>
+    <t>Rung 8B, row 6 (Venue 97, kp-spirits-ii)</t>
+  </si>
+  <si>
+    <t>Business-analyst bypassed the sanctioned tool entirely, twice, using raw inline openpyxl to read the Data Dictionary directly during the KP Spirits II parent-venue fork — first attempt also chained with cd &amp;&amp;, second attempt dropped the chaining but still used inline openpyxl instead of the sanctioned script. Both denied live.</t>
+  </si>
+  <si>
+    <t>business-analyst.md's tool-script section only ever documented writing data/audit_log.xlsx — it never listed dump-data-dictionary (or read-row, --help, dump-audit-log) as sanctioned, and its inline-Python prohibition was scoped to writing the Audit Log only, never to reading, and never to docs/data-dictionary.xlsx at all.</t>
+  </si>
+  <si>
+    <t>business-analyst.md rewritten to mirror worker.md's fuller treatment — explicit sanctioned-command list, inline-Python prohibition widened to reading as well as writing, across both data/audit_log.xlsx and docs/data-dictionary.xlsx. Shipped in PR #11 (andrews-driving-services).</t>
+  </si>
+  <si>
+    <t>A subagent can be using several tool-script subcommands successfully in practice while none of them are actually documented as sanctioned in its own file — the gap only surfaces when it reaches for something the same undocumented territory doesn't cover as gracefully.</t>
+  </si>
+  <si>
+    <t>Rung 8B, row 15 (Venue 106, tim-smith)</t>
+  </si>
+  <si>
+    <t>Business-analyst's next fork attempt correctly targeted the sanctioned script (ads_xlsx_tool.py --help) but chained it with ls ... &amp;&amp; and used an absolute Windows path. Denied live with a steer toward the bare sanctioned shape; self-corrected clean on the next attempt.</t>
+  </si>
+  <si>
+    <t>Same underlying gap as Entry 38 — business-analyst.md never stated the exact invocation shape applies to reads, only demonstrated it in the audit-log-write context.</t>
+  </si>
+  <si>
+    <t>Same fix, same PR (#11, andrews-driving-services) — the exact-shape requirement is now stated explicitly alongside the newly-listed read commands, not only in the audit-log-write section.</t>
+  </si>
+  <si>
+    <t>A correction that fixes the target (right script) without also fixing the shape (chaining, absolute path) isn't a full correction — both matter independently, and a live steer that only addresses one can still leave the other in place until it's tested again.</t>
+  </si>
+  <si>
+    <t>Rung 8B (stopped row 22/25)</t>
+  </si>
+  <si>
+    <t>Rung 8B hard-stopped at row 22/25 when the session's WebSearch budget hit 200/200 — correctly classified and handled as a tool-capability-gap Explicit Hard-Stop, not a defect. 21 of 25 target rows completed before the stop.</t>
+  </si>
+  <si>
+    <t>Not applicable — an observed environment-level resource ceiling, not a defect. STOP-CAPS already covers turn cap, time cap, and stall, but nothing previously named WebSearch budget as a real, distinct constraint on achievable N.</t>
+  </si>
+  <si>
+    <t>No infra/mechanism change — the existing tool-capability-gap/Explicit Hard-Stop machinery already handled this correctly the moment it was hit. Goal Card bumped to v12 (troy-kb PR #6) to report WebSearch calls used going forward, alongside turns and wall-clock, so future N choices can be informed by the empirical calls-per-row rate (~9–10 calls/row observed this rung).</t>
+  </si>
+  <si>
+    <t>A stop condition working exactly as designed can still reveal a gap one level up — in this case, in what gets reported and tracked afterward, not in what stopped the rung.</t>
+  </si>
+  <si>
+    <t>Aug 29 2026 (informed by Rung 8B, Aug 20 — Audit Log Entries #7, #8)</t>
+  </si>
+  <si>
+    <t>Data Dictionary Fields 7 &amp; 8</t>
+  </si>
+  <si>
+    <t>Data Dictionary's Field 7 (Parent Venue) and Field 8 (Venue-Within-Venue Notes) — Instructions for RowBuilder rewritten and added, directly informed by Audit Log Entries #7 (KP Spirits II parent-venue fork) and #8 (Tim Smith Spirits location fork), plus the live Bold Rock Carter Mountain / Bold Rock Hard Cider example (Venues 111 and 49).</t>
+  </si>
+  <si>
+    <t>Field 7's original instruction ("Human might be required...") predated the loop's demonstrated ability to resolve most parent-venue forks itself via read-row, and Field 8 had no Instructions for RowBuilder at all — a real gap surfaced only once two live forks needed to reason through it from scratch.</t>
+  </si>
+  <si>
+    <t>Troy rewrote both fields' Instructions for RowBuilder directly in Excel (his own source-controlled domain) — Field 7 now distinguishes "parent exists" (business-analyst resolves via read-row) from "parent doesn't exist anywhere" (genuine human/stop-and-report case), cites the 196-venue list's observed stability, and gives two worked examples (Bold Rock Hard Cider/Carter Mountain; Winery at Kindred Pointe/KP Spirits II). Field 8 now covers property-level context, not just literal containment, with an explicit "Parent Venue is the central documentation of the relationship" tiebreaker. Companion worker.md update (PR #12, andrews-driving-services) extends worker's sanctioned reference-row fallback to the four rows these examples cite.</t>
+  </si>
+  <si>
+    <t>A field's own worked examples, once they exist, can become live citations elsewhere in the same architecture (worker's reference-row list) — Data Dictionary edits and subagent-file edits aren't always independent once real examples are in play.</t>
   </si>
 </sst>
 </file>
@@ -1008,7 +1071,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -2063,7 +2126,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="179.4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="179.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -2090,6 +2153,122 @@
       </c>
       <c r="I38" s="4" t="s">
         <v>200</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="137.69999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="112.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
+        <v>39</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="155.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
+        <v>40</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="300" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <v>41</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>